<commit_message>
working on result folder
</commit_message>
<xml_diff>
--- a/result folder/Candidate List.xlsx
+++ b/result folder/Candidate List.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git_repository\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git_repository\result folder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B65A7DA3-7E72-4412-84DD-97F951F7F50B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09301007-CF4E-43DF-9FDD-863F5F81B770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4764" yWindow="1944" windowWidth="17280" windowHeight="8880" xr2:uid="{49515CB9-8875-40E7-9298-620E27316FC0}"/>
+    <workbookView xWindow="5460" yWindow="2640" windowWidth="17280" windowHeight="8880" xr2:uid="{49515CB9-8875-40E7-9298-620E27316FC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="36">
   <si>
     <t>VR Meditation Candidate list</t>
   </si>
@@ -65,9 +65,6 @@
     <t>Male</t>
   </si>
   <si>
-    <t>Stress(01)</t>
-  </si>
-  <si>
     <t>conventional</t>
   </si>
   <si>
@@ -120,6 +117,33 @@
   </si>
   <si>
     <t>ali asghar</t>
+  </si>
+  <si>
+    <t>abdul shahbaz</t>
+  </si>
+  <si>
+    <t>Asad Tahseen</t>
+  </si>
+  <si>
+    <t>Naveen</t>
+  </si>
+  <si>
+    <t>raza ansari</t>
+  </si>
+  <si>
+    <t>conventonal</t>
+  </si>
+  <si>
+    <t>zahra abbasi</t>
+  </si>
+  <si>
+    <t>Ouroosha Butt</t>
+  </si>
+  <si>
+    <t>shah muhammad</t>
+  </si>
+  <si>
+    <t>ahmed hussain</t>
   </si>
 </sst>
 </file>
@@ -581,10 +605,10 @@
         <v>6</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -600,11 +624,11 @@
       <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="1">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="G3" s="2">
         <v>0.20833333333333334</v>
@@ -618,7 +642,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1">
         <v>30</v>
@@ -630,7 +654,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G4" s="2">
         <v>0.20833333333333334</v>
@@ -644,7 +668,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C5" s="1">
         <v>24</v>
@@ -656,7 +680,7 @@
         <v>2</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G5" s="2">
         <v>0.20833333333333334</v>
@@ -670,7 +694,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="1">
         <v>34</v>
@@ -682,7 +706,7 @@
         <v>3</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G6" s="2">
         <v>0.20833333333333334</v>
@@ -696,7 +720,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" s="1">
         <v>31</v>
@@ -708,7 +732,7 @@
         <v>4</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G7" s="2">
         <v>0.20833333333333334</v>
@@ -722,7 +746,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1">
         <v>32</v>
@@ -734,7 +758,7 @@
         <v>5</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G8" s="2">
         <v>0.20833333333333334</v>
@@ -748,7 +772,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C9" s="1">
         <v>33</v>
@@ -760,7 +784,7 @@
         <v>6</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G9" s="2">
         <v>0.20833333333333334</v>
@@ -774,19 +798,19 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10" s="1">
         <v>30</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E10" s="1">
         <v>7</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G10" s="2">
         <v>0.20833333333333334</v>
@@ -795,7 +819,7 @@
         <v>0.20833333333333334</v>
       </c>
       <c r="I10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -803,19 +827,19 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11" s="1">
         <v>29</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E11" s="1">
         <v>8</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G11" s="2">
         <v>0.20833333333333334</v>
@@ -829,19 +853,19 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C12" s="1">
         <v>28</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E12" s="1">
         <v>9</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G12" s="2">
         <v>0.20833333333333334</v>
@@ -855,104 +879,234 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C13" s="1">
         <v>36</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E13" s="1">
         <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G13" s="2">
         <v>0.20833333333333334</v>
       </c>
-      <c r="H13" s="1"/>
+      <c r="H13" s="2">
+        <v>0.24722222222222223</v>
+      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
+      <c r="A14" s="1">
+        <v>12</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="1">
+        <v>32</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="1">
+        <v>11</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0.21319444444444444</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
+      <c r="A15" s="1">
+        <v>13</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="1">
+        <v>30</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="1">
+        <v>12</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0.25624999999999998</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
+      <c r="A16" s="1">
+        <v>14</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="1">
+        <v>29</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="1">
+        <v>13</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H16" s="2">
+        <v>0.24930555555555556</v>
+      </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
+      <c r="A17" s="1">
+        <v>15</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="1">
+        <v>28</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="1">
+        <v>14</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0.20833333333333334</v>
+      </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
+      <c r="A18" s="1">
+        <v>16</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="1">
+        <v>29</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" s="1">
+        <v>15</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H18" s="2">
+        <v>0.24444444444444444</v>
+      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
+      <c r="A19" s="1">
+        <v>17</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="1">
+        <v>30</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" s="1">
+        <v>16</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H19" s="2">
+        <v>0.37152777777777779</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
+      <c r="A20" s="1">
+        <v>18</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="1">
+        <v>32</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" s="1">
+        <v>17</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H20" s="2">
+        <v>0.20833333333333334</v>
+      </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
+      <c r="A21" s="1">
+        <v>19</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="1">
+        <v>28</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="1">
+        <v>18</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G21" s="2">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H21" s="2">
+        <v>0.20833333333333334</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>

</xml_diff>

<commit_message>
Data cleaning of stress and conventional method
</commit_message>
<xml_diff>
--- a/result folder/Candidate List.xlsx
+++ b/result folder/Candidate List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git_repository\result folder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09301007-CF4E-43DF-9FDD-863F5F81B770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{781D2B3A-4467-4E52-99CA-B9A0423084D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5460" yWindow="2640" windowWidth="17280" windowHeight="8880" xr2:uid="{49515CB9-8875-40E7-9298-620E27316FC0}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{49515CB9-8875-40E7-9298-620E27316FC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="37">
   <si>
     <t>VR Meditation Candidate list</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>ahmed hussain</t>
+  </si>
+  <si>
+    <t>farhaj kazmi</t>
   </si>
 </sst>
 </file>
@@ -1109,14 +1112,30 @@
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
+      <c r="A22" s="1">
+        <v>20</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="1">
+        <v>28</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="1">
+        <v>19</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G22" s="2">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H22" s="2">
+        <v>0.20902777777777778</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>

</xml_diff>

<commit_message>
changes suggested by supervisor
</commit_message>
<xml_diff>
--- a/result folder/Candidate List.xlsx
+++ b/result folder/Candidate List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git_repository\result folder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{781D2B3A-4467-4E52-99CA-B9A0423084D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFB507BC-6701-4188-B106-18D3E0EF58FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{49515CB9-8875-40E7-9298-620E27316FC0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="49">
   <si>
     <t>VR Meditation Candidate list</t>
   </si>
@@ -147,22 +147,50 @@
   </si>
   <si>
     <t>farhaj kazmi</t>
+  </si>
+  <si>
+    <t>touseef</t>
+  </si>
+  <si>
+    <t>muhammad awais</t>
+  </si>
+  <si>
+    <t>zain</t>
+  </si>
+  <si>
+    <t>meditates daily and also performed AI guided VR meditation</t>
+  </si>
+  <si>
+    <t>sajjad</t>
+  </si>
+  <si>
+    <t>Ikhlaq</t>
+  </si>
+  <si>
+    <t>done both meditation</t>
+  </si>
+  <si>
+    <t>adil butt</t>
+  </si>
+  <si>
+    <t>situ</t>
+  </si>
+  <si>
+    <t>bilal</t>
+  </si>
+  <si>
+    <t>sarah musvi</t>
+  </si>
+  <si>
+    <t>syed ajaz haider</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -173,6 +201,21 @@
       <b/>
       <i/>
       <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -214,19 +257,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -562,263 +608,263 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4E912F7-D1AB-4F16-B8D6-61886A3A073D}">
-  <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I46"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="2">
         <v>29</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="1">
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H3" s="2">
+      <c r="G3" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H3" s="3">
         <v>0.10138888888888889</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <v>30</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="1">
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2">
         <v>1</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H4" s="2">
+      <c r="G4" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H4" s="3">
         <v>0.36805555555555558</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <v>24</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="1">
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2">
         <v>2</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H5" s="2">
+      <c r="G5" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H5" s="3">
         <v>0.36666666666666664</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="2">
         <v>34</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="1">
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2">
         <v>3</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H6" s="2">
+      <c r="G6" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H6" s="3">
         <v>0.17708333333333334</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="2">
         <v>31</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="1">
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2">
         <v>4</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H7" s="2">
+      <c r="G7" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H7" s="3">
         <v>0.24861111111111112</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>6</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="2">
         <v>32</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="1">
+      <c r="D8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2">
         <v>5</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H8" s="2">
+      <c r="G8" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H8" s="3">
         <v>0.1673611111111111</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>7</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="2">
         <v>33</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="1">
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2">
         <v>6</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G9" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H9" s="2">
+      <c r="G9" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H9" s="3">
         <v>0.20555555555555555</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>8</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="A10" s="2">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="2">
         <v>30</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>7</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G10" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H10" s="2">
+      <c r="G10" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H10" s="3">
         <v>0.20833333333333334</v>
       </c>
       <c r="I10" t="s">
@@ -826,351 +872,726 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>9</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="2">
         <v>29</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="1">
-        <v>8</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="E11" s="2">
+        <v>8</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G11" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H11" s="2">
+      <c r="G11" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H11" s="3">
         <v>0.20833333333333334</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>10</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="2">
         <v>28</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>9</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G12" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H12" s="2">
+      <c r="G12" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H12" s="3">
         <v>0.20902777777777778</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>11</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="2">
         <v>36</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>10</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H13" s="2">
+      <c r="G13" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H13" s="3">
         <v>0.24722222222222223</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>12</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="2">
         <v>32</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>11</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H14" s="2">
+      <c r="G14" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H14" s="3">
         <v>0.21319444444444444</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>13</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="2">
         <v>30</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>12</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F15" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H15" s="2">
+      <c r="G15" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H15" s="3">
         <v>0.25624999999999998</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>14</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="2">
         <v>29</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="1">
+      <c r="D16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="2">
         <v>13</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H16" s="2">
+      <c r="G16" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H16" s="3">
         <v>0.24930555555555556</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="1">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
         <v>15</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="2">
         <v>28</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E17" s="1">
+      <c r="D17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="2">
         <v>14</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F17" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="G17" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H17" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="1">
+      <c r="G17" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H17" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="2">
         <v>29</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>15</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G18" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H18" s="2">
+      <c r="G18" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H18" s="3">
         <v>0.24444444444444444</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="1">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
         <v>17</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="2">
         <v>30</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>16</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G19" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H19" s="2">
+      <c r="G19" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H19" s="3">
         <v>0.37152777777777779</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="1">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
         <v>18</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="2">
         <v>32</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>17</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F20" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G20" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H20" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="1">
+      <c r="G20" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H20" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
         <v>19</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" s="2">
         <v>28</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E21" s="1">
+      <c r="D21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="2">
         <v>18</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F21" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G21" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H21" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="1">
+      <c r="G21" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H21" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
         <v>20</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22" s="2">
         <v>28</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22" s="1">
+      <c r="D22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="2">
         <v>19</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="F22" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G22" s="2">
-        <v>0.20833333333333334</v>
-      </c>
-      <c r="H22" s="2">
+      <c r="G22" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H22" s="3">
         <v>0.20902777777777778</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" s="2">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="2">
+        <v>29</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" s="2">
+        <v>20</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H23" s="3">
+        <v>0.20902777777777778</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="2">
+        <v>32</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E24" s="2">
+        <v>21</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H24" s="3">
+        <v>0.24930555555555556</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
+        <v>23</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="2">
+        <v>27</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25" s="2">
+        <v>22</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G25" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H25" s="3">
+        <v>0.16041666666666668</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="2">
+        <v>33</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E26" s="2">
+        <v>23</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G26" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H26" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="I26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
+        <v>25</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="2">
+        <v>32</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" s="2">
+        <v>24</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G27" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H27" s="3">
+        <v>0.16319444444444445</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>26</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" s="2">
+        <v>25</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="2">
+        <v>25</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H28" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="I28" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" s="2">
+        <v>27</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="2">
+        <v>28</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E29" s="2">
+        <v>26</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G29" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H29" s="3">
+        <v>0.15902777777777777</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" s="2">
+        <v>28</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" s="2">
+        <v>29</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E30" s="2">
+        <v>27</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G30" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H30" s="3">
+        <v>0.25277777777777777</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" s="2">
+        <v>29</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" s="2">
+        <v>24</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" s="2">
+        <v>28</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G31" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H31" s="3">
+        <v>0.17291666666666666</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" s="2">
+        <v>30</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C32" s="2">
+        <v>27</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E32" s="2">
+        <v>29</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G32" s="3">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="H32" s="3">
+        <v>0.24861111111111112</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="2">
+        <v>31</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
codes for the data cleaning and plotting graphs
</commit_message>
<xml_diff>
--- a/result folder/Candidate List.xlsx
+++ b/result folder/Candidate List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git_repository\result folder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFB507BC-6701-4188-B106-18D3E0EF58FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF65F098-2FDF-4B25-8335-668CE1070BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{49515CB9-8875-40E7-9298-620E27316FC0}"/>
+    <workbookView xWindow="4248" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{49515CB9-8875-40E7-9298-620E27316FC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="51">
   <si>
     <t>VR Meditation Candidate list</t>
   </si>
@@ -183,6 +183,12 @@
   </si>
   <si>
     <t>syed ajaz haider</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>low</t>
   </si>
 </sst>
 </file>
@@ -674,7 +680,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="2">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>9</v>
@@ -700,7 +706,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="2">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>13</v>
@@ -710,6 +716,9 @@
       </c>
       <c r="H4" s="3">
         <v>0.36805555555555558</v>
+      </c>
+      <c r="I4" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -726,7 +735,7 @@
         <v>8</v>
       </c>
       <c r="E5" s="2">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>13</v>
@@ -736,6 +745,9 @@
       </c>
       <c r="H5" s="3">
         <v>0.36666666666666664</v>
+      </c>
+      <c r="I5" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -752,7 +764,7 @@
         <v>8</v>
       </c>
       <c r="E6" s="2">
-        <v>3</v>
+        <v>103</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>9</v>
@@ -778,7 +790,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="2">
-        <v>4</v>
+        <v>104</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>13</v>
@@ -788,6 +800,9 @@
       </c>
       <c r="H7" s="3">
         <v>0.24861111111111112</v>
+      </c>
+      <c r="I7" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -804,7 +819,7 @@
         <v>8</v>
       </c>
       <c r="E8" s="2">
-        <v>5</v>
+        <v>105</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>9</v>
@@ -830,7 +845,7 @@
         <v>8</v>
       </c>
       <c r="E9" s="2">
-        <v>6</v>
+        <v>106</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>20</v>
@@ -840,6 +855,9 @@
       </c>
       <c r="H9" s="3">
         <v>0.20555555555555555</v>
+      </c>
+      <c r="I9" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -856,7 +874,7 @@
         <v>22</v>
       </c>
       <c r="E10" s="2">
-        <v>7</v>
+        <v>107</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>9</v>
@@ -885,7 +903,7 @@
         <v>22</v>
       </c>
       <c r="E11" s="2">
-        <v>8</v>
+        <v>108</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>9</v>
@@ -911,7 +929,7 @@
         <v>15</v>
       </c>
       <c r="E12" s="2">
-        <v>9</v>
+        <v>109</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>20</v>
@@ -921,6 +939,9 @@
       </c>
       <c r="H12" s="3">
         <v>0.20902777777777778</v>
+      </c>
+      <c r="I12" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -937,7 +958,7 @@
         <v>15</v>
       </c>
       <c r="E13" s="2">
-        <v>10</v>
+        <v>110</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>20</v>
@@ -947,6 +968,9 @@
       </c>
       <c r="H13" s="3">
         <v>0.24722222222222223</v>
+      </c>
+      <c r="I13" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -963,7 +987,7 @@
         <v>15</v>
       </c>
       <c r="E14" s="2">
-        <v>11</v>
+        <v>111</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>13</v>
@@ -973,6 +997,9 @@
       </c>
       <c r="H14" s="3">
         <v>0.21319444444444444</v>
+      </c>
+      <c r="I14" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -989,7 +1016,7 @@
         <v>15</v>
       </c>
       <c r="E15" s="2">
-        <v>12</v>
+        <v>112</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>13</v>
@@ -999,6 +1026,9 @@
       </c>
       <c r="H15" s="3">
         <v>0.25624999999999998</v>
+      </c>
+      <c r="I15" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
@@ -1015,7 +1045,7 @@
         <v>8</v>
       </c>
       <c r="E16" s="2">
-        <v>13</v>
+        <v>113</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>13</v>
@@ -1025,6 +1055,9 @@
       </c>
       <c r="H16" s="3">
         <v>0.24930555555555556</v>
+      </c>
+      <c r="I16" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
@@ -1041,7 +1074,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="2">
-        <v>14</v>
+        <v>114</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>31</v>
@@ -1067,7 +1100,7 @@
         <v>22</v>
       </c>
       <c r="E18" s="2">
-        <v>15</v>
+        <v>115</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>20</v>
@@ -1077,6 +1110,9 @@
       </c>
       <c r="H18" s="3">
         <v>0.24444444444444444</v>
+      </c>
+      <c r="I18" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
@@ -1093,7 +1129,7 @@
         <v>22</v>
       </c>
       <c r="E19" s="2">
-        <v>16</v>
+        <v>116</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>20</v>
@@ -1103,6 +1139,9 @@
       </c>
       <c r="H19" s="3">
         <v>0.37152777777777779</v>
+      </c>
+      <c r="I19" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
@@ -1119,7 +1158,7 @@
         <v>15</v>
       </c>
       <c r="E20" s="2">
-        <v>17</v>
+        <v>117</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>9</v>
@@ -1145,7 +1184,7 @@
         <v>8</v>
       </c>
       <c r="E21" s="2">
-        <v>18</v>
+        <v>118</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>9</v>
@@ -1171,7 +1210,7 @@
         <v>8</v>
       </c>
       <c r="E22" s="2">
-        <v>19</v>
+        <v>119</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>9</v>
@@ -1197,7 +1236,7 @@
         <v>15</v>
       </c>
       <c r="E23" s="2">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>13</v>
@@ -1207,6 +1246,9 @@
       </c>
       <c r="H23" s="3">
         <v>0.20902777777777778</v>
+      </c>
+      <c r="I23" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
@@ -1223,7 +1265,7 @@
         <v>15</v>
       </c>
       <c r="E24" s="2">
-        <v>21</v>
+        <v>121</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>13</v>
@@ -1233,6 +1275,9 @@
       </c>
       <c r="H24" s="3">
         <v>0.24930555555555556</v>
+      </c>
+      <c r="I24" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
@@ -1249,7 +1294,7 @@
         <v>8</v>
       </c>
       <c r="E25" s="2">
-        <v>22</v>
+        <v>122</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>20</v>
@@ -1259,6 +1304,9 @@
       </c>
       <c r="H25" s="3">
         <v>0.16041666666666668</v>
+      </c>
+      <c r="I25" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
@@ -1275,7 +1323,7 @@
         <v>15</v>
       </c>
       <c r="E26" s="2">
-        <v>23</v>
+        <v>123</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>9</v>
@@ -1304,7 +1352,7 @@
         <v>15</v>
       </c>
       <c r="E27" s="2">
-        <v>24</v>
+        <v>124</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>20</v>
@@ -1314,6 +1362,9 @@
       </c>
       <c r="H27" s="3">
         <v>0.16319444444444445</v>
+      </c>
+      <c r="I27" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
@@ -1330,7 +1381,7 @@
         <v>8</v>
       </c>
       <c r="E28" s="2">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>9</v>
@@ -1359,7 +1410,7 @@
         <v>8</v>
       </c>
       <c r="E29" s="2">
-        <v>26</v>
+        <v>126</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>20</v>
@@ -1369,6 +1420,9 @@
       </c>
       <c r="H29" s="3">
         <v>0.15902777777777777</v>
+      </c>
+      <c r="I29" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
@@ -1385,7 +1439,7 @@
         <v>22</v>
       </c>
       <c r="E30" s="2">
-        <v>27</v>
+        <v>127</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>20</v>
@@ -1395,6 +1449,9 @@
       </c>
       <c r="H30" s="3">
         <v>0.25277777777777777</v>
+      </c>
+      <c r="I30" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
@@ -1411,7 +1468,7 @@
         <v>8</v>
       </c>
       <c r="E31" s="2">
-        <v>28</v>
+        <v>128</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>20</v>
@@ -1421,6 +1478,9 @@
       </c>
       <c r="H31" s="3">
         <v>0.17291666666666666</v>
+      </c>
+      <c r="I31" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
@@ -1437,7 +1497,7 @@
         <v>22</v>
       </c>
       <c r="E32" s="2">
-        <v>29</v>
+        <v>129</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>20</v>
@@ -1447,6 +1507,9 @@
       </c>
       <c r="H32" s="3">
         <v>0.24861111111111112</v>
+      </c>
+      <c r="I32" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>